<commit_message>
Auto saved by Logseq
</commit_message>
<xml_diff>
--- a/assets/dbt_macro_second_day_1763444063100_0.xlsx
+++ b/assets/dbt_macro_second_day_1763444063100_0.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\htetoo\notes\logseq\assets\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{84ED2403-2E78-4A48-BF19-02E97B7C5120}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8742CD0A-701E-4721-BA0B-5CB1D0B90947}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="14016" xr2:uid="{9838F717-2D2E-4437-A497-9E5F6DC1BC32}"/>
   </bookViews>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="90" uniqueCount="57">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="109" uniqueCount="72">
   <si>
     <t>left</t>
   </si>
@@ -151,9 +151,6 @@
     <t>character varying(1500)</t>
   </si>
   <si>
-    <t>trn_amount numeric(38,4) ENCODE az64,</t>
-  </si>
-  <si>
     <t>character varying(10)</t>
   </si>
   <si>
@@ -166,9 +163,6 @@
     <t>numeric(38,9)</t>
   </si>
   <si>
-    <t>CREATE TABLE report.fn_daily_loan_drawdown_acc_trn (</t>
-  </si>
-  <si>
     <t>)</t>
   </si>
   <si>
@@ -181,31 +175,82 @@
     <t>trn_category character varying(100) ENCODE lzo COLLATE case_sensitive,</t>
   </si>
   <si>
-    <t>acc_no character varying(80) ENCODE lzo COLLATE case_sensitive,</t>
-  </si>
-  <si>
-    <t>cust_no character varying(27) ENCODE lzo COLLATE case_sensitive,</t>
-  </si>
-  <si>
     <t>cust_segment character varying(35) ENCODE lzo COLLATE case_sensitive,</t>
   </si>
   <si>
-    <t>week_num character varying(25) ENCODE lzo COLLATE case_sensitive,</t>
-  </si>
-  <si>
-    <t>counter_change_amount numeric(38,4) ENCODE az64,</t>
-  </si>
-  <si>
-    <t>without_counter_change_amount numeric(38,4) ENCODE az64,</t>
-  </si>
-  <si>
-    <t>amount_type character varying(10) ENCODE lzo COLLATE case_sensitive</t>
-  </si>
-  <si>
     <t>character varying(80)</t>
   </si>
   <si>
     <t>character varying(25)</t>
+  </si>
+  <si>
+    <t>trn_branch character varying(12) ENCODE lzo COLLATE case_sensitive,</t>
+  </si>
+  <si>
+    <t>trn_township character varying(255) ENCODE lzo COLLATE case_sensitive,</t>
+  </si>
+  <si>
+    <t>trn_division character varying(255) ENCODE lzo COLLATE case_sensitive,</t>
+  </si>
+  <si>
+    <t>trn_territory character varying(255) ENCODE lzo COLLATE case_sensitive,</t>
+  </si>
+  <si>
+    <t>acc_class character varying(18) ENCODE lzo COLLATE case_sensitive,</t>
+  </si>
+  <si>
+    <t>product_group character varying(16383) ENCODE lzo COLLATE case_sensitive,</t>
+  </si>
+  <si>
+    <t>product_category character varying(16383) ENCODE lzo COLLATE case_sensitive,</t>
+  </si>
+  <si>
+    <t>cust_type character varying(10) ENCODE lzo COLLATE case_sensitive,</t>
+  </si>
+  <si>
+    <t>acc_branch character varying(12) ENCODE lzo COLLATE case_sensitive,</t>
+  </si>
+  <si>
+    <t>acc_township character varying(255) ENCODE lzo COLLATE case_sensitive,</t>
+  </si>
+  <si>
+    <t>acc_division character varying(255) ENCODE lzo COLLATE case_sensitive,</t>
+  </si>
+  <si>
+    <t>acc_territory character varying(255) ENCODE lzo COLLATE case_sensitive,</t>
+  </si>
+  <si>
+    <t>trn_amt_tier character varying(21) ENCODE lzo COLLATE case_sensitive,</t>
+  </si>
+  <si>
+    <t>no_of_accounts bigint ENCODE az64,</t>
+  </si>
+  <si>
+    <t>trn_count bigint ENCODE az64,</t>
+  </si>
+  <si>
+    <t>character varying(255)</t>
+  </si>
+  <si>
+    <t>character varying(16383)</t>
+  </si>
+  <si>
+    <t>CREATE TABLE report.dbu_monthly_trn_history (</t>
+  </si>
+  <si>
+    <t>in/out character varying(7) ENCODE lzo COLLATE case_sensitive,</t>
+  </si>
+  <si>
+    <t>business_sector character varying(4000) ENCODE lzo COLLATE case_sensitive,</t>
+  </si>
+  <si>
+    <t>business_industry_type character varying(4000) ENCODE lzo COLLATE case_sensitive,</t>
+  </si>
+  <si>
+    <t>business_sub_industry character varying(4000) ENCODE lzo COLLATE case_sensitive,</t>
+  </si>
+  <si>
+    <t>trn_amount numeric(38,4) ENCODE az64</t>
   </si>
 </sst>
 </file>
@@ -558,7 +603,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{37C584A1-B989-4751-AD72-3D826A76C96E}">
-  <dimension ref="A1:N36"/>
+  <dimension ref="A1:N39"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="58.109375" bestFit="1" customWidth="1"/>
@@ -593,7 +638,7 @@
     </row>
     <row r="2" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
-        <v>43</v>
+        <v>66</v>
       </c>
       <c r="C2" t="str">
         <f>LEFT(A2,FIND(" ",A2)-1)</f>
@@ -643,19 +688,19 @@
     </row>
     <row r="4" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
-        <v>46</v>
+        <v>49</v>
       </c>
       <c r="C4" t="str">
         <f t="shared" si="0"/>
-        <v>trn_group</v>
+        <v>trn_branch</v>
       </c>
       <c r="D4" t="str">
         <f t="shared" ref="D4:D6" si="1">LEFT(A4,FIND("ENCODE",A4)-2)</f>
-        <v>trn_group character varying(50)</v>
+        <v>trn_branch character varying(12)</v>
       </c>
       <c r="E4" t="str">
         <f t="shared" ref="E4:E32" si="2">RIGHT(D4,LEN(D4)-FIND(" ",D4))</f>
-        <v>character varying(50)</v>
+        <v>character varying(12)</v>
       </c>
       <c r="F4" t="str">
         <f t="shared" ref="F4:F6" si="3">VLOOKUP(E4,M:N,2,FALSE)</f>
@@ -663,7 +708,7 @@
       </c>
       <c r="G4" t="str">
         <f t="shared" ref="G4:G6" si="4">F4&amp;C4&amp;","</f>
-        <v>null as trn_group,</v>
+        <v>null as trn_branch,</v>
       </c>
       <c r="M4" t="s">
         <v>6</v>
@@ -674,19 +719,19 @@
     </row>
     <row r="5" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
-        <v>47</v>
+        <v>50</v>
       </c>
       <c r="C5" t="str">
         <f t="shared" si="0"/>
-        <v>trn_category</v>
+        <v>trn_township</v>
       </c>
       <c r="D5" t="str">
         <f t="shared" si="1"/>
-        <v>trn_category character varying(100)</v>
+        <v>trn_township character varying(255)</v>
       </c>
       <c r="E5" t="str">
         <f t="shared" si="2"/>
-        <v>character varying(100)</v>
+        <v>character varying(255)</v>
       </c>
       <c r="F5" t="str">
         <f t="shared" si="3"/>
@@ -694,7 +739,7 @@
       </c>
       <c r="G5" t="str">
         <f t="shared" si="4"/>
-        <v>null as trn_category,</v>
+        <v>null as trn_township,</v>
       </c>
       <c r="M5" t="s">
         <v>7</v>
@@ -705,19 +750,19 @@
     </row>
     <row r="6" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
-        <v>48</v>
+        <v>51</v>
       </c>
       <c r="C6" t="str">
         <f t="shared" si="0"/>
-        <v>acc_no</v>
+        <v>trn_division</v>
       </c>
       <c r="D6" t="str">
         <f t="shared" si="1"/>
-        <v>acc_no character varying(80)</v>
+        <v>trn_division character varying(255)</v>
       </c>
       <c r="E6" t="str">
         <f t="shared" si="2"/>
-        <v>character varying(80)</v>
+        <v>character varying(255)</v>
       </c>
       <c r="F6" t="str">
         <f t="shared" si="3"/>
@@ -725,7 +770,7 @@
       </c>
       <c r="G6" t="str">
         <f t="shared" si="4"/>
-        <v>null as acc_no,</v>
+        <v>null as trn_division,</v>
       </c>
       <c r="M6" t="s">
         <v>8</v>
@@ -736,19 +781,19 @@
     </row>
     <row r="7" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
-        <v>49</v>
+        <v>52</v>
       </c>
       <c r="C7" t="str">
         <f t="shared" si="0"/>
-        <v>cust_no</v>
+        <v>trn_territory</v>
       </c>
       <c r="D7" t="str">
         <f t="shared" ref="D7" si="5">LEFT(A7,FIND("ENCODE",A7)-2)</f>
-        <v>cust_no character varying(27)</v>
+        <v>trn_territory character varying(255)</v>
       </c>
       <c r="E7" t="str">
         <f t="shared" si="2"/>
-        <v>character varying(27)</v>
+        <v>character varying(255)</v>
       </c>
       <c r="F7" t="str">
         <f t="shared" ref="F7" si="6">VLOOKUP(E7,M:N,2,FALSE)</f>
@@ -756,7 +801,7 @@
       </c>
       <c r="G7" t="str">
         <f t="shared" ref="G7" si="7">F7&amp;C7&amp;","</f>
-        <v>null as cust_no,</v>
+        <v>null as trn_territory,</v>
       </c>
       <c r="M7" t="s">
         <v>9</v>
@@ -767,19 +812,19 @@
     </row>
     <row r="8" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
-        <v>50</v>
+        <v>67</v>
       </c>
       <c r="C8" t="str">
         <f t="shared" si="0"/>
-        <v>cust_segment</v>
+        <v>in/out</v>
       </c>
       <c r="D8" t="str">
         <f t="shared" ref="D8" si="8">LEFT(A8,FIND("ENCODE",A8)-2)</f>
-        <v>cust_segment character varying(35)</v>
+        <v>in/out character varying(7)</v>
       </c>
       <c r="E8" t="str">
         <f t="shared" si="2"/>
-        <v>character varying(35)</v>
+        <v>character varying(7)</v>
       </c>
       <c r="F8" t="str">
         <f t="shared" ref="F8" si="9">VLOOKUP(E8,M:N,2,FALSE)</f>
@@ -787,7 +832,7 @@
       </c>
       <c r="G8" t="str">
         <f t="shared" ref="G8" si="10">F8&amp;C8&amp;","</f>
-        <v>null as cust_segment,</v>
+        <v>null as in/out,</v>
       </c>
       <c r="M8" t="s">
         <v>10</v>
@@ -798,19 +843,19 @@
     </row>
     <row r="9" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="C9" t="str">
         <f t="shared" si="0"/>
-        <v>week_num</v>
+        <v>acc_class</v>
       </c>
       <c r="D9" t="str">
         <f t="shared" ref="D9:D32" si="11">LEFT(A9,FIND("ENCODE",A9)-2)</f>
-        <v>week_num character varying(25)</v>
+        <v>acc_class character varying(18)</v>
       </c>
       <c r="E9" t="str">
         <f t="shared" si="2"/>
-        <v>character varying(25)</v>
+        <v>character varying(18)</v>
       </c>
       <c r="F9" t="str">
         <f t="shared" ref="F9:F32" si="12">VLOOKUP(E9,M:N,2,FALSE)</f>
@@ -818,7 +863,7 @@
       </c>
       <c r="G9" t="str">
         <f t="shared" ref="G9:G32" si="13">F9&amp;C9&amp;","</f>
-        <v>null as week_num,</v>
+        <v>null as acc_class,</v>
       </c>
       <c r="M9" t="s">
         <v>11</v>
@@ -829,27 +874,27 @@
     </row>
     <row r="10" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
-        <v>38</v>
+        <v>54</v>
       </c>
       <c r="C10" t="str">
         <f t="shared" si="0"/>
-        <v>trn_amount</v>
+        <v>product_group</v>
       </c>
       <c r="D10" t="str">
         <f t="shared" si="11"/>
-        <v>trn_amount numeric(38,4)</v>
+        <v>product_group character varying(16383)</v>
       </c>
       <c r="E10" t="str">
         <f t="shared" si="2"/>
-        <v>numeric(38,4)</v>
+        <v>character varying(16383)</v>
       </c>
       <c r="F10" t="str">
         <f t="shared" si="12"/>
-        <v xml:space="preserve">0 as </v>
+        <v xml:space="preserve">null as </v>
       </c>
       <c r="G10" t="str">
         <f t="shared" si="13"/>
-        <v>0 as trn_amount,</v>
+        <v>null as product_group,</v>
       </c>
       <c r="M10" t="s">
         <v>12</v>
@@ -860,27 +905,27 @@
     </row>
     <row r="11" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
-        <v>52</v>
+        <v>55</v>
       </c>
       <c r="C11" t="str">
         <f t="shared" si="0"/>
-        <v>counter_change_amount</v>
+        <v>product_category</v>
       </c>
       <c r="D11" t="str">
         <f t="shared" si="11"/>
-        <v>counter_change_amount numeric(38,4)</v>
+        <v>product_category character varying(16383)</v>
       </c>
       <c r="E11" t="str">
         <f t="shared" si="2"/>
-        <v>numeric(38,4)</v>
+        <v>character varying(16383)</v>
       </c>
       <c r="F11" t="str">
         <f t="shared" si="12"/>
-        <v xml:space="preserve">0 as </v>
+        <v xml:space="preserve">null as </v>
       </c>
       <c r="G11" t="str">
         <f t="shared" si="13"/>
-        <v>0 as counter_change_amount,</v>
+        <v>null as product_category,</v>
       </c>
       <c r="M11" t="s">
         <v>17</v>
@@ -891,27 +936,27 @@
     </row>
     <row r="12" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
-        <v>53</v>
+        <v>56</v>
       </c>
       <c r="C12" t="str">
         <f t="shared" si="0"/>
-        <v>without_counter_change_amount</v>
+        <v>cust_type</v>
       </c>
       <c r="D12" t="str">
         <f t="shared" si="11"/>
-        <v>without_counter_change_amount numeric(38,4)</v>
+        <v>cust_type character varying(10)</v>
       </c>
       <c r="E12" t="str">
         <f t="shared" si="2"/>
-        <v>numeric(38,4)</v>
+        <v>character varying(10)</v>
       </c>
       <c r="F12" t="str">
         <f t="shared" si="12"/>
-        <v xml:space="preserve">0 as </v>
+        <v xml:space="preserve">null as </v>
       </c>
       <c r="G12" t="str">
         <f t="shared" si="13"/>
-        <v>0 as without_counter_change_amount,</v>
+        <v>null as cust_type,</v>
       </c>
       <c r="M12" t="s">
         <v>18</v>
@@ -922,19 +967,19 @@
     </row>
     <row r="13" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
-        <v>54</v>
+        <v>46</v>
       </c>
       <c r="C13" t="str">
         <f t="shared" si="0"/>
-        <v>amount_type</v>
+        <v>cust_segment</v>
       </c>
       <c r="D13" t="str">
         <f t="shared" si="11"/>
-        <v>amount_type character varying(10)</v>
+        <v>cust_segment character varying(35)</v>
       </c>
       <c r="E13" t="str">
         <f t="shared" si="2"/>
-        <v>character varying(10)</v>
+        <v>character varying(35)</v>
       </c>
       <c r="F13" t="str">
         <f t="shared" si="12"/>
@@ -942,7 +987,7 @@
       </c>
       <c r="G13" t="str">
         <f t="shared" si="13"/>
-        <v>null as amount_type,</v>
+        <v>null as cust_segment,</v>
       </c>
       <c r="M13" t="s">
         <v>19</v>
@@ -953,27 +998,27 @@
     </row>
     <row r="14" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
-        <v>44</v>
-      </c>
-      <c r="C14" t="e">
-        <f t="shared" si="0"/>
-        <v>#VALUE!</v>
-      </c>
-      <c r="D14" t="e">
-        <f t="shared" si="11"/>
-        <v>#VALUE!</v>
-      </c>
-      <c r="E14" t="e">
-        <f t="shared" si="2"/>
-        <v>#VALUE!</v>
-      </c>
-      <c r="F14" t="e">
-        <f t="shared" si="12"/>
-        <v>#VALUE!</v>
-      </c>
-      <c r="G14" t="e">
-        <f t="shared" si="13"/>
-        <v>#VALUE!</v>
+        <v>68</v>
+      </c>
+      <c r="C14" t="str">
+        <f t="shared" si="0"/>
+        <v>business_sector</v>
+      </c>
+      <c r="D14" t="str">
+        <f t="shared" si="11"/>
+        <v>business_sector character varying(4000)</v>
+      </c>
+      <c r="E14" t="str">
+        <f t="shared" si="2"/>
+        <v>character varying(4000)</v>
+      </c>
+      <c r="F14" t="str">
+        <f t="shared" si="12"/>
+        <v xml:space="preserve">null as </v>
+      </c>
+      <c r="G14" t="str">
+        <f t="shared" si="13"/>
+        <v>null as business_sector,</v>
       </c>
       <c r="M14" t="s">
         <v>20</v>
@@ -984,27 +1029,27 @@
     </row>
     <row r="15" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
-        <v>45</v>
+        <v>69</v>
       </c>
       <c r="C15" t="str">
         <f t="shared" si="0"/>
-        <v>DISTSTYLE</v>
-      </c>
-      <c r="D15" t="e">
-        <f t="shared" si="11"/>
-        <v>#VALUE!</v>
-      </c>
-      <c r="E15" t="e">
-        <f t="shared" si="2"/>
-        <v>#VALUE!</v>
-      </c>
-      <c r="F15" t="e">
-        <f t="shared" si="12"/>
-        <v>#VALUE!</v>
-      </c>
-      <c r="G15" t="e">
-        <f t="shared" si="13"/>
-        <v>#VALUE!</v>
+        <v>business_industry_type</v>
+      </c>
+      <c r="D15" t="str">
+        <f t="shared" si="11"/>
+        <v>business_industry_type character varying(4000)</v>
+      </c>
+      <c r="E15" t="str">
+        <f t="shared" si="2"/>
+        <v>character varying(4000)</v>
+      </c>
+      <c r="F15" t="str">
+        <f t="shared" si="12"/>
+        <v xml:space="preserve">null as </v>
+      </c>
+      <c r="G15" t="str">
+        <f t="shared" si="13"/>
+        <v>null as business_industry_type,</v>
       </c>
       <c r="M15" t="s">
         <v>22</v>
@@ -1014,25 +1059,28 @@
       </c>
     </row>
     <row r="16" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="C16" t="e">
-        <f t="shared" si="0"/>
-        <v>#VALUE!</v>
-      </c>
-      <c r="D16" t="e">
-        <f t="shared" si="11"/>
-        <v>#VALUE!</v>
-      </c>
-      <c r="E16" t="e">
-        <f t="shared" si="2"/>
-        <v>#VALUE!</v>
-      </c>
-      <c r="F16" t="e">
-        <f t="shared" si="12"/>
-        <v>#VALUE!</v>
-      </c>
-      <c r="G16" t="e">
-        <f t="shared" si="13"/>
-        <v>#VALUE!</v>
+      <c r="A16" t="s">
+        <v>70</v>
+      </c>
+      <c r="C16" t="str">
+        <f t="shared" si="0"/>
+        <v>business_sub_industry</v>
+      </c>
+      <c r="D16" t="str">
+        <f t="shared" si="11"/>
+        <v>business_sub_industry character varying(4000)</v>
+      </c>
+      <c r="E16" t="str">
+        <f t="shared" si="2"/>
+        <v>character varying(4000)</v>
+      </c>
+      <c r="F16" t="str">
+        <f t="shared" si="12"/>
+        <v xml:space="preserve">null as </v>
+      </c>
+      <c r="G16" t="str">
+        <f t="shared" si="13"/>
+        <v>null as business_sub_industry,</v>
       </c>
       <c r="M16" t="s">
         <v>23</v>
@@ -1041,26 +1089,29 @@
         <v>13</v>
       </c>
     </row>
-    <row r="17" spans="3:14" x14ac:dyDescent="0.3">
-      <c r="C17" t="e">
-        <f t="shared" si="0"/>
-        <v>#VALUE!</v>
-      </c>
-      <c r="D17" t="e">
-        <f t="shared" si="11"/>
-        <v>#VALUE!</v>
-      </c>
-      <c r="E17" t="e">
-        <f t="shared" si="2"/>
-        <v>#VALUE!</v>
-      </c>
-      <c r="F17" t="e">
-        <f t="shared" si="12"/>
-        <v>#VALUE!</v>
-      </c>
-      <c r="G17" t="e">
-        <f t="shared" si="13"/>
-        <v>#VALUE!</v>
+    <row r="17" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A17" t="s">
+        <v>44</v>
+      </c>
+      <c r="C17" t="str">
+        <f t="shared" si="0"/>
+        <v>trn_group</v>
+      </c>
+      <c r="D17" t="str">
+        <f t="shared" si="11"/>
+        <v>trn_group character varying(50)</v>
+      </c>
+      <c r="E17" t="str">
+        <f t="shared" si="2"/>
+        <v>character varying(50)</v>
+      </c>
+      <c r="F17" t="str">
+        <f t="shared" si="12"/>
+        <v xml:space="preserve">null as </v>
+      </c>
+      <c r="G17" t="str">
+        <f t="shared" si="13"/>
+        <v>null as trn_group,</v>
       </c>
       <c r="M17" t="s">
         <v>24</v>
@@ -1069,26 +1120,29 @@
         <v>13</v>
       </c>
     </row>
-    <row r="18" spans="3:14" x14ac:dyDescent="0.3">
-      <c r="C18" t="e">
-        <f t="shared" si="0"/>
-        <v>#VALUE!</v>
-      </c>
-      <c r="D18" t="e">
-        <f t="shared" si="11"/>
-        <v>#VALUE!</v>
-      </c>
-      <c r="E18" t="e">
-        <f t="shared" si="2"/>
-        <v>#VALUE!</v>
-      </c>
-      <c r="F18" t="e">
-        <f t="shared" si="12"/>
-        <v>#VALUE!</v>
-      </c>
-      <c r="G18" t="e">
-        <f t="shared" si="13"/>
-        <v>#VALUE!</v>
+    <row r="18" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A18" t="s">
+        <v>45</v>
+      </c>
+      <c r="C18" t="str">
+        <f t="shared" si="0"/>
+        <v>trn_category</v>
+      </c>
+      <c r="D18" t="str">
+        <f t="shared" si="11"/>
+        <v>trn_category character varying(100)</v>
+      </c>
+      <c r="E18" t="str">
+        <f t="shared" si="2"/>
+        <v>character varying(100)</v>
+      </c>
+      <c r="F18" t="str">
+        <f t="shared" si="12"/>
+        <v xml:space="preserve">null as </v>
+      </c>
+      <c r="G18" t="str">
+        <f t="shared" si="13"/>
+        <v>null as trn_category,</v>
       </c>
       <c r="M18" t="s">
         <v>25</v>
@@ -1097,26 +1151,29 @@
         <v>13</v>
       </c>
     </row>
-    <row r="19" spans="3:14" x14ac:dyDescent="0.3">
-      <c r="C19" t="e">
-        <f t="shared" si="0"/>
-        <v>#VALUE!</v>
-      </c>
-      <c r="D19" t="e">
-        <f t="shared" si="11"/>
-        <v>#VALUE!</v>
-      </c>
-      <c r="E19" t="e">
-        <f t="shared" si="2"/>
-        <v>#VALUE!</v>
-      </c>
-      <c r="F19" t="e">
-        <f t="shared" si="12"/>
-        <v>#VALUE!</v>
-      </c>
-      <c r="G19" t="e">
-        <f t="shared" si="13"/>
-        <v>#VALUE!</v>
+    <row r="19" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A19" t="s">
+        <v>57</v>
+      </c>
+      <c r="C19" t="str">
+        <f t="shared" si="0"/>
+        <v>acc_branch</v>
+      </c>
+      <c r="D19" t="str">
+        <f t="shared" si="11"/>
+        <v>acc_branch character varying(12)</v>
+      </c>
+      <c r="E19" t="str">
+        <f t="shared" si="2"/>
+        <v>character varying(12)</v>
+      </c>
+      <c r="F19" t="str">
+        <f t="shared" si="12"/>
+        <v xml:space="preserve">null as </v>
+      </c>
+      <c r="G19" t="str">
+        <f t="shared" si="13"/>
+        <v>null as acc_branch,</v>
       </c>
       <c r="M19" t="s">
         <v>26</v>
@@ -1125,26 +1182,29 @@
         <v>13</v>
       </c>
     </row>
-    <row r="20" spans="3:14" x14ac:dyDescent="0.3">
-      <c r="C20" t="e">
-        <f t="shared" si="0"/>
-        <v>#VALUE!</v>
-      </c>
-      <c r="D20" t="e">
-        <f t="shared" si="11"/>
-        <v>#VALUE!</v>
-      </c>
-      <c r="E20" t="e">
-        <f t="shared" si="2"/>
-        <v>#VALUE!</v>
-      </c>
-      <c r="F20" t="e">
-        <f t="shared" si="12"/>
-        <v>#VALUE!</v>
-      </c>
-      <c r="G20" t="e">
-        <f t="shared" si="13"/>
-        <v>#VALUE!</v>
+    <row r="20" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A20" t="s">
+        <v>58</v>
+      </c>
+      <c r="C20" t="str">
+        <f t="shared" si="0"/>
+        <v>acc_township</v>
+      </c>
+      <c r="D20" t="str">
+        <f t="shared" si="11"/>
+        <v>acc_township character varying(255)</v>
+      </c>
+      <c r="E20" t="str">
+        <f t="shared" si="2"/>
+        <v>character varying(255)</v>
+      </c>
+      <c r="F20" t="str">
+        <f t="shared" si="12"/>
+        <v xml:space="preserve">null as </v>
+      </c>
+      <c r="G20" t="str">
+        <f t="shared" si="13"/>
+        <v>null as acc_township,</v>
       </c>
       <c r="M20" t="s">
         <v>27</v>
@@ -1153,26 +1213,29 @@
         <v>13</v>
       </c>
     </row>
-    <row r="21" spans="3:14" x14ac:dyDescent="0.3">
-      <c r="C21" t="e">
-        <f t="shared" si="0"/>
-        <v>#VALUE!</v>
-      </c>
-      <c r="D21" t="e">
-        <f t="shared" si="11"/>
-        <v>#VALUE!</v>
-      </c>
-      <c r="E21" t="e">
-        <f t="shared" si="2"/>
-        <v>#VALUE!</v>
-      </c>
-      <c r="F21" t="e">
-        <f t="shared" si="12"/>
-        <v>#VALUE!</v>
-      </c>
-      <c r="G21" t="e">
-        <f t="shared" si="13"/>
-        <v>#VALUE!</v>
+    <row r="21" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A21" t="s">
+        <v>59</v>
+      </c>
+      <c r="C21" t="str">
+        <f t="shared" si="0"/>
+        <v>acc_division</v>
+      </c>
+      <c r="D21" t="str">
+        <f t="shared" si="11"/>
+        <v>acc_division character varying(255)</v>
+      </c>
+      <c r="E21" t="str">
+        <f t="shared" si="2"/>
+        <v>character varying(255)</v>
+      </c>
+      <c r="F21" t="str">
+        <f t="shared" si="12"/>
+        <v xml:space="preserve">null as </v>
+      </c>
+      <c r="G21" t="str">
+        <f t="shared" si="13"/>
+        <v>null as acc_division,</v>
       </c>
       <c r="M21" t="s">
         <v>28</v>
@@ -1181,26 +1244,29 @@
         <v>13</v>
       </c>
     </row>
-    <row r="22" spans="3:14" x14ac:dyDescent="0.3">
-      <c r="C22" t="e">
-        <f t="shared" si="0"/>
-        <v>#VALUE!</v>
-      </c>
-      <c r="D22" t="e">
-        <f t="shared" si="11"/>
-        <v>#VALUE!</v>
-      </c>
-      <c r="E22" t="e">
-        <f t="shared" si="2"/>
-        <v>#VALUE!</v>
-      </c>
-      <c r="F22" t="e">
-        <f t="shared" si="12"/>
-        <v>#VALUE!</v>
-      </c>
-      <c r="G22" t="e">
-        <f t="shared" si="13"/>
-        <v>#VALUE!</v>
+    <row r="22" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A22" t="s">
+        <v>60</v>
+      </c>
+      <c r="C22" t="str">
+        <f t="shared" si="0"/>
+        <v>acc_territory</v>
+      </c>
+      <c r="D22" t="str">
+        <f t="shared" si="11"/>
+        <v>acc_territory character varying(255)</v>
+      </c>
+      <c r="E22" t="str">
+        <f t="shared" si="2"/>
+        <v>character varying(255)</v>
+      </c>
+      <c r="F22" t="str">
+        <f t="shared" si="12"/>
+        <v xml:space="preserve">null as </v>
+      </c>
+      <c r="G22" t="str">
+        <f t="shared" si="13"/>
+        <v>null as acc_territory,</v>
       </c>
       <c r="M22" t="s">
         <v>29</v>
@@ -1209,26 +1275,29 @@
         <v>13</v>
       </c>
     </row>
-    <row r="23" spans="3:14" x14ac:dyDescent="0.3">
-      <c r="C23" t="e">
-        <f t="shared" si="0"/>
-        <v>#VALUE!</v>
-      </c>
-      <c r="D23" t="e">
-        <f t="shared" si="11"/>
-        <v>#VALUE!</v>
-      </c>
-      <c r="E23" t="e">
-        <f t="shared" si="2"/>
-        <v>#VALUE!</v>
-      </c>
-      <c r="F23" t="e">
-        <f t="shared" si="12"/>
-        <v>#VALUE!</v>
-      </c>
-      <c r="G23" t="e">
-        <f t="shared" si="13"/>
-        <v>#VALUE!</v>
+    <row r="23" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A23" t="s">
+        <v>61</v>
+      </c>
+      <c r="C23" t="str">
+        <f t="shared" si="0"/>
+        <v>trn_amt_tier</v>
+      </c>
+      <c r="D23" t="str">
+        <f t="shared" si="11"/>
+        <v>trn_amt_tier character varying(21)</v>
+      </c>
+      <c r="E23" t="str">
+        <f t="shared" si="2"/>
+        <v>character varying(21)</v>
+      </c>
+      <c r="F23" t="str">
+        <f t="shared" si="12"/>
+        <v xml:space="preserve">null as </v>
+      </c>
+      <c r="G23" t="str">
+        <f t="shared" si="13"/>
+        <v>null as trn_amt_tier,</v>
       </c>
       <c r="M23" t="s">
         <v>30</v>
@@ -1237,26 +1306,29 @@
         <v>13</v>
       </c>
     </row>
-    <row r="24" spans="3:14" x14ac:dyDescent="0.3">
-      <c r="C24" t="e">
-        <f t="shared" si="0"/>
-        <v>#VALUE!</v>
-      </c>
-      <c r="D24" t="e">
-        <f t="shared" si="11"/>
-        <v>#VALUE!</v>
-      </c>
-      <c r="E24" t="e">
-        <f t="shared" si="2"/>
-        <v>#VALUE!</v>
-      </c>
-      <c r="F24" t="e">
-        <f t="shared" si="12"/>
-        <v>#VALUE!</v>
-      </c>
-      <c r="G24" t="e">
-        <f t="shared" si="13"/>
-        <v>#VALUE!</v>
+    <row r="24" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A24" t="s">
+        <v>62</v>
+      </c>
+      <c r="C24" t="str">
+        <f t="shared" si="0"/>
+        <v>no_of_accounts</v>
+      </c>
+      <c r="D24" t="str">
+        <f t="shared" si="11"/>
+        <v>no_of_accounts bigint</v>
+      </c>
+      <c r="E24" t="str">
+        <f t="shared" si="2"/>
+        <v>bigint</v>
+      </c>
+      <c r="F24" t="str">
+        <f t="shared" si="12"/>
+        <v xml:space="preserve">0 as </v>
+      </c>
+      <c r="G24" t="str">
+        <f t="shared" si="13"/>
+        <v>0 as no_of_accounts,</v>
       </c>
       <c r="M24" t="s">
         <v>31</v>
@@ -1265,26 +1337,29 @@
         <v>14</v>
       </c>
     </row>
-    <row r="25" spans="3:14" x14ac:dyDescent="0.3">
-      <c r="C25" t="e">
-        <f t="shared" si="0"/>
-        <v>#VALUE!</v>
-      </c>
-      <c r="D25" t="e">
-        <f t="shared" si="11"/>
-        <v>#VALUE!</v>
-      </c>
-      <c r="E25" t="e">
-        <f t="shared" si="2"/>
-        <v>#VALUE!</v>
-      </c>
-      <c r="F25" t="e">
-        <f t="shared" si="12"/>
-        <v>#VALUE!</v>
-      </c>
-      <c r="G25" t="e">
-        <f t="shared" si="13"/>
-        <v>#VALUE!</v>
+    <row r="25" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A25" t="s">
+        <v>63</v>
+      </c>
+      <c r="C25" t="str">
+        <f t="shared" si="0"/>
+        <v>trn_count</v>
+      </c>
+      <c r="D25" t="str">
+        <f t="shared" si="11"/>
+        <v>trn_count bigint</v>
+      </c>
+      <c r="E25" t="str">
+        <f t="shared" si="2"/>
+        <v>bigint</v>
+      </c>
+      <c r="F25" t="str">
+        <f t="shared" si="12"/>
+        <v xml:space="preserve">0 as </v>
+      </c>
+      <c r="G25" t="str">
+        <f t="shared" si="13"/>
+        <v>0 as trn_count,</v>
       </c>
       <c r="M25" t="s">
         <v>32</v>
@@ -1293,26 +1368,29 @@
         <v>13</v>
       </c>
     </row>
-    <row r="26" spans="3:14" x14ac:dyDescent="0.3">
-      <c r="C26" t="e">
-        <f t="shared" si="0"/>
-        <v>#VALUE!</v>
-      </c>
-      <c r="D26" t="e">
-        <f t="shared" si="11"/>
-        <v>#VALUE!</v>
-      </c>
-      <c r="E26" t="e">
-        <f t="shared" si="2"/>
-        <v>#VALUE!</v>
-      </c>
-      <c r="F26" t="e">
-        <f t="shared" si="12"/>
-        <v>#VALUE!</v>
-      </c>
-      <c r="G26" t="e">
-        <f t="shared" si="13"/>
-        <v>#VALUE!</v>
+    <row r="26" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A26" t="s">
+        <v>71</v>
+      </c>
+      <c r="C26" t="str">
+        <f t="shared" si="0"/>
+        <v>trn_amount</v>
+      </c>
+      <c r="D26" t="str">
+        <f t="shared" si="11"/>
+        <v>trn_amount numeric(38,4)</v>
+      </c>
+      <c r="E26" t="str">
+        <f t="shared" si="2"/>
+        <v>numeric(38,4)</v>
+      </c>
+      <c r="F26" t="str">
+        <f t="shared" si="12"/>
+        <v xml:space="preserve">0 as </v>
+      </c>
+      <c r="G26" t="str">
+        <f t="shared" si="13"/>
+        <v>0 as trn_amount,</v>
       </c>
       <c r="M26" t="s">
         <v>33</v>
@@ -1321,7 +1399,10 @@
         <v>13</v>
       </c>
     </row>
-    <row r="27" spans="3:14" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A27" t="s">
+        <v>42</v>
+      </c>
       <c r="C27" t="e">
         <f t="shared" si="0"/>
         <v>#VALUE!</v>
@@ -1349,10 +1430,13 @@
         <v>14</v>
       </c>
     </row>
-    <row r="28" spans="3:14" x14ac:dyDescent="0.3">
-      <c r="C28" t="e">
-        <f t="shared" si="0"/>
-        <v>#VALUE!</v>
+    <row r="28" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A28" t="s">
+        <v>43</v>
+      </c>
+      <c r="C28" t="str">
+        <f t="shared" si="0"/>
+        <v>DISTSTYLE</v>
       </c>
       <c r="D28" t="e">
         <f t="shared" si="11"/>
@@ -1377,7 +1461,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="29" spans="3:14" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:14" x14ac:dyDescent="0.3">
       <c r="C29" t="e">
         <f t="shared" si="0"/>
         <v>#VALUE!</v>
@@ -1405,7 +1489,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="30" spans="3:14" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:14" x14ac:dyDescent="0.3">
       <c r="C30" t="e">
         <f t="shared" si="0"/>
         <v>#VALUE!</v>
@@ -1433,7 +1517,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="31" spans="3:14" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:14" x14ac:dyDescent="0.3">
       <c r="C31" t="e">
         <f t="shared" si="0"/>
         <v>#VALUE!</v>
@@ -1455,70 +1539,134 @@
         <v>#VALUE!</v>
       </c>
       <c r="M31" t="s">
+        <v>38</v>
+      </c>
+      <c r="N31" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="32" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="C32" t="e">
+        <f t="shared" si="0"/>
+        <v>#VALUE!</v>
+      </c>
+      <c r="D32" t="e">
+        <f t="shared" si="11"/>
+        <v>#VALUE!</v>
+      </c>
+      <c r="E32" t="e">
+        <f t="shared" si="2"/>
+        <v>#VALUE!</v>
+      </c>
+      <c r="F32" t="e">
+        <f t="shared" si="12"/>
+        <v>#VALUE!</v>
+      </c>
+      <c r="G32" t="e">
+        <f t="shared" si="13"/>
+        <v>#VALUE!</v>
+      </c>
+      <c r="M32" t="s">
         <v>39</v>
       </c>
-      <c r="N31" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="32" spans="3:14" x14ac:dyDescent="0.3">
-      <c r="C32" t="e">
-        <f t="shared" si="0"/>
-        <v>#VALUE!</v>
-      </c>
-      <c r="D32" t="e">
-        <f t="shared" si="11"/>
-        <v>#VALUE!</v>
-      </c>
-      <c r="E32" t="e">
-        <f t="shared" si="2"/>
-        <v>#VALUE!</v>
-      </c>
-      <c r="F32" t="e">
-        <f t="shared" si="12"/>
-        <v>#VALUE!</v>
-      </c>
-      <c r="G32" t="e">
-        <f t="shared" si="13"/>
-        <v>#VALUE!</v>
-      </c>
-      <c r="M32" t="s">
+      <c r="N32" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="33" spans="3:14" x14ac:dyDescent="0.3">
+      <c r="C33" t="e">
+        <f t="shared" ref="C33:C34" si="14">LEFT(A33,FIND(" ",A33)-1)</f>
+        <v>#VALUE!</v>
+      </c>
+      <c r="D33" t="e">
+        <f t="shared" ref="D33:D34" si="15">LEFT(A33,FIND("ENCODE",A33)-2)</f>
+        <v>#VALUE!</v>
+      </c>
+      <c r="E33" t="e">
+        <f t="shared" ref="E33:E34" si="16">RIGHT(D33,LEN(D33)-FIND(" ",D33))</f>
+        <v>#VALUE!</v>
+      </c>
+      <c r="F33" t="e">
+        <f t="shared" ref="F33:F34" si="17">VLOOKUP(E33,M:N,2,FALSE)</f>
+        <v>#VALUE!</v>
+      </c>
+      <c r="G33" t="e">
+        <f t="shared" ref="G33:G34" si="18">F33&amp;C33&amp;","</f>
+        <v>#VALUE!</v>
+      </c>
+      <c r="M33" t="s">
         <v>40</v>
       </c>
-      <c r="N32" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="33" spans="13:14" x14ac:dyDescent="0.3">
-      <c r="M33" t="s">
+      <c r="N33" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="34" spans="3:14" x14ac:dyDescent="0.3">
+      <c r="C34" t="e">
+        <f t="shared" si="14"/>
+        <v>#VALUE!</v>
+      </c>
+      <c r="D34" t="e">
+        <f t="shared" si="15"/>
+        <v>#VALUE!</v>
+      </c>
+      <c r="E34" t="e">
+        <f t="shared" si="16"/>
+        <v>#VALUE!</v>
+      </c>
+      <c r="F34" t="e">
+        <f t="shared" si="17"/>
+        <v>#VALUE!</v>
+      </c>
+      <c r="G34" t="e">
+        <f t="shared" si="18"/>
+        <v>#VALUE!</v>
+      </c>
+      <c r="M34" t="s">
         <v>41</v>
-      </c>
-      <c r="N33" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="34" spans="13:14" x14ac:dyDescent="0.3">
-      <c r="M34" t="s">
-        <v>42</v>
       </c>
       <c r="N34" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="35" spans="13:14" x14ac:dyDescent="0.3">
+    <row r="35" spans="3:14" x14ac:dyDescent="0.3">
       <c r="M35" t="s">
-        <v>55</v>
+        <v>47</v>
       </c>
       <c r="N35" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="36" spans="13:14" x14ac:dyDescent="0.3">
+    <row r="36" spans="3:14" x14ac:dyDescent="0.3">
       <c r="M36" t="s">
-        <v>56</v>
+        <v>48</v>
       </c>
       <c r="N36" t="s">
         <v>13</v>
+      </c>
+    </row>
+    <row r="37" spans="3:14" x14ac:dyDescent="0.3">
+      <c r="M37" t="s">
+        <v>64</v>
+      </c>
+      <c r="N37" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="38" spans="3:14" x14ac:dyDescent="0.3">
+      <c r="M38" t="s">
+        <v>65</v>
+      </c>
+      <c r="N38" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="39" spans="3:14" x14ac:dyDescent="0.3">
+      <c r="M39" t="s">
+        <v>10</v>
+      </c>
+      <c r="N39" t="s">
+        <v>14</v>
       </c>
     </row>
   </sheetData>

</xml_diff>